<commit_message>
Add no-code deck route: EY deck skeleton and Deck_Tokens tab
Skeleton deck on the EY template with placeholders; master template
gains a formula-driven Deck_Tokens tab. Prompt 8 now uses Copilot in
PowerPoint or Find and Replace instead of Python.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JceH5MqRn93y3Fzok3yEHi
</commit_message>
<xml_diff>
--- a/copilot-nature-agent/Nature_Opportunity_Master_Template.xlsx
+++ b/copilot-nature-agent/Nature_Opportunity_Master_Template.xlsx
@@ -21,7 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slide_Content" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Log" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck_Tokens" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Log" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5350,7 +5351,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Paste Copilot Step 7 output here (Key | Value). build_deck.py reads this tab plus the Scoring tab to build the EY deck.</t>
+          <t>Paste Copilot Step 7 output here (Key | Value). The Deck_Tokens tab turns this and the Scoring tab into placeholder values for the EY deck skeleton.</t>
         </is>
       </c>
     </row>
@@ -5439,20 +5440,20 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>s1_stat1_value</t>
+          <t>stat1</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>e.g. £60.0bn</t>
+          <t>Headline figure, e.g. £60.0bn</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>s1_stat1_label</t>
+          <t>stat1_text</t>
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
@@ -5465,7 +5466,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>s1_stat2_value</t>
+          <t>stat2</t>
         </is>
       </c>
       <c r="B12" s="6" t="n"/>
@@ -5478,7 +5479,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>s1_stat2_label</t>
+          <t>stat2_text</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
@@ -5491,7 +5492,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>s1_stat3_value</t>
+          <t>stat3</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
@@ -5504,7 +5505,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>s1_stat3_label</t>
+          <t>stat3_text</t>
         </is>
       </c>
       <c r="B15" s="6" t="n"/>
@@ -6053,6 +6054,1436 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B129"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Placeholder values for Nature_Deck_Skeleton_EY.pptx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>All formulas. Copy columns A:B (rows 5 down) into Copilot in PowerPoint (Prompt 8), or use them for Find and Replace (Ctrl+H).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>High + Medium rows</t>
+        </is>
+      </c>
+      <c r="B3" s="16">
+        <f>MIN(12,COUNTIF(Scoring!$K$5:$K$19,"High")+COUNTIF(Scoring!$K$5:$K$19,"Medium"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>{{cover_title}}</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>IF(Slide_Content!$B$5="","",Slide_Content!$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>{{cover_date}}</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>IF(Slide_Content!$B$6="","",Slide_Content!$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>{{client_name}}</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>IF(Slide_Content!$B$7="","",Slide_Content!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_title}}</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>IF(Slide_Content!$B$8="","",Slide_Content!$B$8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_section}}</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>IF(Slide_Content!$B$9="","",Slide_Content!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>{{stat1}}</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>IF(Slide_Content!$B$10="","",Slide_Content!$B$10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>{{stat1_text}}</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>IF(Slide_Content!$B$11="","",Slide_Content!$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>{{stat2}}</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>IF(Slide_Content!$B$12="","",Slide_Content!$B$12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>{{stat2_text}}</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>IF(Slide_Content!$B$13="","",Slide_Content!$B$13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>{{stat3}}</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>IF(Slide_Content!$B$14="","",Slide_Content!$B$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>{{stat3_text}}</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>IF(Slide_Content!$B$15="","",Slide_Content!$B$15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_context}}</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>IF(Slide_Content!$B$16="","",Slide_Content!$B$16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_finding1}}</t>
+        </is>
+      </c>
+      <c r="B17" s="8">
+        <f>IF(Slide_Content!$B$17="","",Slide_Content!$B$17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_finding2}}</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>IF(Slide_Content!$B$18="","",Slide_Content!$B$18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_finding3}}</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>IF(Slide_Content!$B$19="","",Slide_Content!$B$19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_priorities}}</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>IF(Slide_Content!$B$20="","",Slide_Content!$B$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_implication}}</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>IF(Slide_Content!$B$21="","",Slide_Content!$B$21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_footnote}}</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>IF(Slide_Content!$B$22="","",Slide_Content!$B$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>{{s1_notes}}</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>IF(Slide_Content!$B$23="","",Slide_Content!$B$23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>{{s2_title}}</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>IF(Slide_Content!$B$24="","",Slide_Content!$B$24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>{{s2_section}}</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>IF(Slide_Content!$B$25="","",Slide_Content!$B$25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>{{s2_low_note}}</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <f>IF(Slide_Content!$B$26="","",Slide_Content!$B$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>{{s2_footnote}}</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>IF(Slide_Content!$B$27="","",Slide_Content!$B$27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>{{s2_notes}}</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <f>IF(Slide_Content!$B$28="","",Slide_Content!$B$28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_title}}</t>
+        </is>
+      </c>
+      <c r="B29" s="8">
+        <f>IF(Slide_Content!$B$29="","",Slide_Content!$B$29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_section}}</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <f>IF(Slide_Content!$B$30="","",Slide_Content!$B$30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card1_title}}</t>
+        </is>
+      </c>
+      <c r="B31" s="8">
+        <f>IF(Slide_Content!$B$31="","",Slide_Content!$B$31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card1_score}}</t>
+        </is>
+      </c>
+      <c r="B32" s="8">
+        <f>IF(Slide_Content!$B$32="","",Slide_Content!$B$32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card1_evidence}}</t>
+        </is>
+      </c>
+      <c r="B33" s="8">
+        <f>IF(Slide_Content!$B$33="","",Slide_Content!$B$33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card1_support}}</t>
+        </is>
+      </c>
+      <c r="B34" s="8">
+        <f>IF(Slide_Content!$B$34="","",Slide_Content!$B$34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card1_output}}</t>
+        </is>
+      </c>
+      <c r="B35" s="8">
+        <f>IF(Slide_Content!$B$35="","",Slide_Content!$B$35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card2_title}}</t>
+        </is>
+      </c>
+      <c r="B36" s="8">
+        <f>IF(Slide_Content!$B$36="","",Slide_Content!$B$36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card2_score}}</t>
+        </is>
+      </c>
+      <c r="B37" s="8">
+        <f>IF(Slide_Content!$B$37="","",Slide_Content!$B$37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card2_evidence}}</t>
+        </is>
+      </c>
+      <c r="B38" s="8">
+        <f>IF(Slide_Content!$B$38="","",Slide_Content!$B$38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card2_support}}</t>
+        </is>
+      </c>
+      <c r="B39" s="8">
+        <f>IF(Slide_Content!$B$39="","",Slide_Content!$B$39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card2_output}}</t>
+        </is>
+      </c>
+      <c r="B40" s="8">
+        <f>IF(Slide_Content!$B$40="","",Slide_Content!$B$40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card3_title}}</t>
+        </is>
+      </c>
+      <c r="B41" s="8">
+        <f>IF(Slide_Content!$B$41="","",Slide_Content!$B$41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card3_score}}</t>
+        </is>
+      </c>
+      <c r="B42" s="8">
+        <f>IF(Slide_Content!$B$42="","",Slide_Content!$B$42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card3_evidence}}</t>
+        </is>
+      </c>
+      <c r="B43" s="8">
+        <f>IF(Slide_Content!$B$43="","",Slide_Content!$B$43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card3_support}}</t>
+        </is>
+      </c>
+      <c r="B44" s="8">
+        <f>IF(Slide_Content!$B$44="","",Slide_Content!$B$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card3_output}}</t>
+        </is>
+      </c>
+      <c r="B45" s="8">
+        <f>IF(Slide_Content!$B$45="","",Slide_Content!$B$45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card4_title}}</t>
+        </is>
+      </c>
+      <c r="B46" s="8">
+        <f>IF(Slide_Content!$B$46="","",Slide_Content!$B$46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card4_score}}</t>
+        </is>
+      </c>
+      <c r="B47" s="8">
+        <f>IF(Slide_Content!$B$47="","",Slide_Content!$B$47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card4_evidence}}</t>
+        </is>
+      </c>
+      <c r="B48" s="8">
+        <f>IF(Slide_Content!$B$48="","",Slide_Content!$B$48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card4_support}}</t>
+        </is>
+      </c>
+      <c r="B49" s="8">
+        <f>IF(Slide_Content!$B$49="","",Slide_Content!$B$49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_card4_output}}</t>
+        </is>
+      </c>
+      <c r="B50" s="8">
+        <f>IF(Slide_Content!$B$50="","",Slide_Content!$B$50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_crosscutting}}</t>
+        </is>
+      </c>
+      <c r="B51" s="8">
+        <f>IF(Slide_Content!$B$51="","",Slide_Content!$B$51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_next1}}</t>
+        </is>
+      </c>
+      <c r="B52" s="8">
+        <f>IF(Slide_Content!$B$52="","",Slide_Content!$B$52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_next2}}</t>
+        </is>
+      </c>
+      <c r="B53" s="8">
+        <f>IF(Slide_Content!$B$53="","",Slide_Content!$B$53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_next3}}</t>
+        </is>
+      </c>
+      <c r="B54" s="8">
+        <f>IF(Slide_Content!$B$54="","",Slide_Content!$B$54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_footnote}}</t>
+        </is>
+      </c>
+      <c r="B55" s="8">
+        <f>IF(Slide_Content!$B$55="","",Slide_Content!$B$55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>{{s3_notes}}</t>
+        </is>
+      </c>
+      <c r="B56" s="8">
+        <f>IF(Slide_Content!$B$56="","",Slide_Content!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>{{1_name}}</t>
+        </is>
+      </c>
+      <c r="B57" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>{{1_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B58" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>{{1_exp}}</t>
+        </is>
+      </c>
+      <c r="B59" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>{{1s}}</t>
+        </is>
+      </c>
+      <c r="B60" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>{{1t}}</t>
+        </is>
+      </c>
+      <c r="B61" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>{{1_evid}}</t>
+        </is>
+      </c>
+      <c r="B62" s="19">
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>{{2_name}}</t>
+        </is>
+      </c>
+      <c r="B63" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>{{2_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B64" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>{{2_exp}}</t>
+        </is>
+      </c>
+      <c r="B65" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>{{2s}}</t>
+        </is>
+      </c>
+      <c r="B66" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>{{2t}}</t>
+        </is>
+      </c>
+      <c r="B67" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>{{2_evid}}</t>
+        </is>
+      </c>
+      <c r="B68" s="19">
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>{{3_name}}</t>
+        </is>
+      </c>
+      <c r="B69" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>{{3_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B70" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>{{3_exp}}</t>
+        </is>
+      </c>
+      <c r="B71" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>{{3s}}</t>
+        </is>
+      </c>
+      <c r="B72" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>{{3t}}</t>
+        </is>
+      </c>
+      <c r="B73" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>{{3_evid}}</t>
+        </is>
+      </c>
+      <c r="B74" s="19">
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>{{4_name}}</t>
+        </is>
+      </c>
+      <c r="B75" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>{{4_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B76" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>{{4_exp}}</t>
+        </is>
+      </c>
+      <c r="B77" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>{{4s}}</t>
+        </is>
+      </c>
+      <c r="B78" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>{{4t}}</t>
+        </is>
+      </c>
+      <c r="B79" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>{{4_evid}}</t>
+        </is>
+      </c>
+      <c r="B80" s="19">
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>{{5_name}}</t>
+        </is>
+      </c>
+      <c r="B81" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>{{5_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B82" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>{{5_exp}}</t>
+        </is>
+      </c>
+      <c r="B83" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>{{5s}}</t>
+        </is>
+      </c>
+      <c r="B84" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>{{5t}}</t>
+        </is>
+      </c>
+      <c r="B85" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>{{5_evid}}</t>
+        </is>
+      </c>
+      <c r="B86" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>{{6_name}}</t>
+        </is>
+      </c>
+      <c r="B87" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>{{6_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B88" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>{{6_exp}}</t>
+        </is>
+      </c>
+      <c r="B89" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>{{6s}}</t>
+        </is>
+      </c>
+      <c r="B90" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>{{6t}}</t>
+        </is>
+      </c>
+      <c r="B91" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>{{6_evid}}</t>
+        </is>
+      </c>
+      <c r="B92" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>{{7_name}}</t>
+        </is>
+      </c>
+      <c r="B93" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>{{7_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B94" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>{{7_exp}}</t>
+        </is>
+      </c>
+      <c r="B95" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>{{7s}}</t>
+        </is>
+      </c>
+      <c r="B96" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>{{7t}}</t>
+        </is>
+      </c>
+      <c r="B97" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>{{7_evid}}</t>
+        </is>
+      </c>
+      <c r="B98" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>{{8_name}}</t>
+        </is>
+      </c>
+      <c r="B99" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>{{8_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B100" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>{{8_exp}}</t>
+        </is>
+      </c>
+      <c r="B101" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>{{8s}}</t>
+        </is>
+      </c>
+      <c r="B102" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>{{8t}}</t>
+        </is>
+      </c>
+      <c r="B103" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>{{8_evid}}</t>
+        </is>
+      </c>
+      <c r="B104" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>{{9_name}}</t>
+        </is>
+      </c>
+      <c r="B105" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>{{9_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B106" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>{{9_exp}}</t>
+        </is>
+      </c>
+      <c r="B107" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>{{9s}}</t>
+        </is>
+      </c>
+      <c r="B108" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>{{9t}}</t>
+        </is>
+      </c>
+      <c r="B109" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>{{9_evid}}</t>
+        </is>
+      </c>
+      <c r="B110" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>{{10_name}}</t>
+        </is>
+      </c>
+      <c r="B111" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>{{10_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B112" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>{{10_exp}}</t>
+        </is>
+      </c>
+      <c r="B113" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>{{10s}}</t>
+        </is>
+      </c>
+      <c r="B114" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>{{10t}}</t>
+        </is>
+      </c>
+      <c r="B115" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>{{10_evid}}</t>
+        </is>
+      </c>
+      <c r="B116" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>{{11_name}}</t>
+        </is>
+      </c>
+      <c r="B117" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>{{11_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B118" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>{{11_exp}}</t>
+        </is>
+      </c>
+      <c r="B119" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>{{11s}}</t>
+        </is>
+      </c>
+      <c r="B120" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>{{11t}}</t>
+        </is>
+      </c>
+      <c r="B121" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>{{11_evid}}</t>
+        </is>
+      </c>
+      <c r="B122" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>{{12_name}}</t>
+        </is>
+      </c>
+      <c r="B123" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>{{12_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B124" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>{{12_exp}}</t>
+        </is>
+      </c>
+      <c r="B125" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>{{12s}}</t>
+        </is>
+      </c>
+      <c r="B126" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>{{12t}}</t>
+        </is>
+      </c>
+      <c r="B127" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>{{12_evid}}</t>
+        </is>
+      </c>
+      <c r="B128" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>{{low_list}}</t>
+        </is>
+      </c>
+      <c r="B129" s="19">
+        <f>IF(1&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(1&lt;15,"  |  ",""),"")&amp;IF(2&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(2&lt;15,"  |  ",""),"")&amp;IF(3&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(3&lt;15,"  |  ",""),"")&amp;IF(4&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(4&lt;15,"  |  ",""),"")&amp;IF(5&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(5&lt;15,"  |  ",""),"")&amp;IF(6&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(6&lt;15,"  |  ",""),"")&amp;IF(7&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(7&lt;15,"  |  ",""),"")&amp;IF(8&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(8&lt;15,"  |  ",""),"")&amp;IF(9&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(9&lt;15,"  |  ",""),"")&amp;IF(10&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(10&lt;15,"  |  ",""),"")&amp;IF(11&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(11&lt;15,"  |  ",""),"")&amp;IF(12&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(12&lt;15,"  |  ",""),"")&amp;IF(13&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(13,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(13,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(13&lt;15,"  |  ",""),"")&amp;IF(14&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(14,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(14,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(14&lt;15,"  |  ",""),"")&amp;IF(15&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(15,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(15,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(15&lt;15,"  |  ",""),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update toolkit to new story and split-slide layouts; archive old decks
Deck skeleton pages 2-3 rebuilt (story-led executive summary,
priority chart vs exposure tiles). Master template gains new
Slide_Content keys, automatic national stats, short names and a
Deck_Chart tab. Guides and methodology document updated. Earlier
LBG decks moved to archive.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JceH5MqRn93y3Fzok3yEHi
</commit_message>
<xml_diff>
--- a/copilot-nature-agent/Nature_Opportunity_Master_Template.xlsx
+++ b/copilot-nature-agent/Nature_Opportunity_Master_Template.xlsx
@@ -22,7 +22,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slide_Content" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck_Tokens" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Log" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deck_Chart" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Log" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5333,7 +5334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5407,642 +5408,1201 @@
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Short client name used on every slide line</t>
+          <t>Full client name for the client line</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>s1_title</t>
+          <t>client_short</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Action title ≤75 characters</t>
+          <t>Short name, e.g. LBG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>s1_section</t>
+          <t>s1_title</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Executive summary</t>
+          <t>Action title ≤75 characters</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>stat1</t>
+          <t>s1_section</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Headline figure, e.g. £60.0bn</t>
+          <t>e.g. Executive summary: why this matters and what we found</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>stat1_text</t>
+          <t>c1_head</t>
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>Signal card heading, ≤7 words, e.g. The UK is putting money behind nature</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>stat2</t>
+          <t>c1_stat</t>
         </is>
       </c>
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>e.g. 4 of 15</t>
+          <t>Leave blank to use the automatic count of national commitments</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>stat2_text</t>
+          <t>c1_stat_text</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>Leave blank for automatic text</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>stat3</t>
+          <t>c1_p1_lead</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>e.g. £70.9bn</t>
+          <t>Bold lead, ≤3 words</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>stat3_text</t>
+          <t>c1_p1</t>
         </is>
       </c>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>s1_context</t>
+          <t>c1_p2_lead</t>
         </is>
       </c>
       <c r="B16" s="6" t="n"/>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>1 sentence</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>s1_finding1</t>
+          <t>c1_p2</t>
         </is>
       </c>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Exposure finding, ≤30 words</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>s1_finding2</t>
+          <t>c1_p3_lead</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Action finding, ≤30 words</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>s1_finding3</t>
+          <t>c1_p3</t>
         </is>
       </c>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Gap finding, ≤30 words</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>s1_priorities</t>
+          <t>c2_head</t>
         </is>
       </c>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>High sub-themes with scores, 1 sentence</t>
+          <t>Rules card heading, ≤7 words</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>s1_implication</t>
+          <t>c2_stat</t>
         </is>
       </c>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>1 sentence</t>
+          <t>Headline figure for regulation or market signal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>s1_footnote</t>
+          <t>c2_stat_text</t>
         </is>
       </c>
       <c r="B22" s="6" t="n"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>1 line</t>
+          <t>≤10 words</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>s1_notes</t>
+          <t>c2_p1_lead</t>
         </is>
       </c>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Sources, one per line</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>s2_title</t>
+          <t>c2_p1</t>
         </is>
       </c>
       <c r="B24" s="6" t="n"/>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Action title ≤75 characters</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>s2_section</t>
+          <t>c2_p2_lead</t>
         </is>
       </c>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Nature priorities ranked by score</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>s2_low_note</t>
+          <t>c2_p2</t>
         </is>
       </c>
       <c r="B26" s="6" t="n"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>1 sentence shown after the Low list</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>s2_footnote</t>
+          <t>c2_p3_lead</t>
         </is>
       </c>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Weights and data caveats, ≤2 lines</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>s2_notes</t>
+          <t>c2_p3</t>
         </is>
       </c>
       <c r="B28" s="6" t="n"/>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Sources, one per line</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>s3_title</t>
+          <t>c3_head</t>
         </is>
       </c>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Action title ≤75 characters</t>
+          <t>Client card heading, ≤7 words</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>s3_section</t>
+          <t>c3_stat</t>
         </is>
       </c>
       <c r="B30" s="6" t="n"/>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>How EY can assist</t>
+          <t>Client headline exposure figure</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>s3_card1_title</t>
+          <t>c3_stat_text</t>
         </is>
       </c>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>≤5 words</t>
+          <t>≤10 words</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>s3_card1_score</t>
+          <t>c3_p1_lead</t>
         </is>
       </c>
       <c r="B32" s="6" t="n"/>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>e.g. 4.5</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>s3_card1_evidence</t>
+          <t>c3_p1</t>
         </is>
       </c>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>s3_card1_support</t>
+          <t>c3_p2_lead</t>
         </is>
       </c>
       <c r="B34" s="6" t="n"/>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>s3_card1_output</t>
+          <t>c3_p2</t>
         </is>
       </c>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>≤10 words</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>s3_card2_title</t>
+          <t>c3_p3_lead</t>
         </is>
       </c>
       <c r="B36" s="6" t="n"/>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>≤5 words</t>
+          <t>Bold lead</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>s3_card2_score</t>
+          <t>c3_p3</t>
         </is>
       </c>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>e.g. 4.5</t>
+          <t>≤8 words</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>s3_card2_evidence</t>
+          <t>s1_found_note</t>
         </is>
       </c>
       <c r="B38" s="6" t="n"/>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>One line under the top-4 priorities, ≤25 words</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>s3_card2_support</t>
+          <t>s1_sowhat</t>
         </is>
       </c>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>One sentence, ≤25 words</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>s3_card2_output</t>
+          <t>s1_footnote</t>
         </is>
       </c>
       <c r="B40" s="6" t="n"/>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>≤10 words</t>
+          <t>Sources, 1–2 lines</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>s3_card3_title</t>
+          <t>s1_notes</t>
         </is>
       </c>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>≤5 words</t>
+          <t>Sources, one per line</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>s3_card3_score</t>
+          <t>s2_title</t>
         </is>
       </c>
       <c r="B42" s="6" t="n"/>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>e.g. 4.5</t>
+          <t>Action title ≤75 characters</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>s3_card3_evidence</t>
+          <t>s2_section</t>
         </is>
       </c>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>e.g. Opportunity priority vs client exposure</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>s3_card3_support</t>
+          <t>exp_unit</t>
         </is>
       </c>
       <c r="B44" s="6" t="n"/>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>e.g. £bn, 31 Dec 2025</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>s3_card3_output</t>
+          <t>t1_value</t>
         </is>
       </c>
       <c r="B45" s="6" t="n"/>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>≤10 words</t>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>s3_card4_title</t>
+          <t>t1_label</t>
         </is>
       </c>
       <c r="B46" s="6" t="n"/>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>≤5 words</t>
+          <t>Sector, ≤6 words</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>s3_card4_score</t>
+          <t>t1_links</t>
         </is>
       </c>
       <c r="B47" s="6" t="n"/>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>e.g. 4.5</t>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>s3_card4_evidence</t>
+          <t>t1_flag</t>
         </is>
       </c>
       <c r="B48" s="6" t="n"/>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>e.g. Nature priority / Not nature priority</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>s3_card4_support</t>
+          <t>t2_value</t>
         </is>
       </c>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>≤20 words</t>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>s3_card4_output</t>
+          <t>t2_label</t>
         </is>
       </c>
       <c r="B50" s="6" t="n"/>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>≤10 words</t>
+          <t>Sector, ≤6 words</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>s3_crosscutting</t>
+          <t>t2_links</t>
         </is>
       </c>
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>1 sentence</t>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>s3_next1</t>
+          <t>t2_flag</t>
         </is>
       </c>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>e.g. Nature priority / Not nature priority</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>s3_next2</t>
+          <t>t3_value</t>
         </is>
       </c>
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>s3_next3</t>
+          <t>t3_label</t>
         </is>
       </c>
       <c r="B54" s="6" t="n"/>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>≤12 words</t>
+          <t>Sector, ≤6 words</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>s3_footnote</t>
+          <t>t3_links</t>
         </is>
       </c>
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>1 line</t>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>s3_notes</t>
+          <t>t3_flag</t>
         </is>
       </c>
       <c r="B56" s="6" t="n"/>
       <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>e.g. Nature priority / Not nature priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>t4_value</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>t4_label</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Sector, ≤6 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>t4_links</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>t4_flag</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>e.g. Nature priority / Not nature priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>t5_value</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>t5_label</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Sector, ≤6 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>t5_links</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>t5_flag</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>e.g. Nature priority / Not nature priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>t6_value</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Exposure figure, e.g. £12.1bn or Not split</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>t6_label</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Sector, ≤6 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>t6_links</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Linked priority ranks, e.g. #3 #4 #7</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>t6_flag</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>e.g. Nature priority / Not nature priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>s2_sowhat</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>One sentence, ≤30 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>s2_footnote</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Weights and sources, ≤2 lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>s2_notes</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Sources, one per line</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>s3_title</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Action title ≤75 characters</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>s3_section</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>How EY can assist</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>s3_card1_title</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>≤5 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>s3_card1_score</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>e.g. 4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>s3_card1_evidence</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>s3_card1_support</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>s3_card1_output</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>≤10 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>s3_card2_title</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>≤5 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>s3_card2_score</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>e.g. 4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>s3_card2_evidence</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>s3_card2_support</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>s3_card2_output</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>≤10 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>s3_card3_title</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>≤5 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>s3_card3_score</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>e.g. 4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>s3_card3_evidence</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>s3_card3_support</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>s3_card3_output</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>≤10 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>s3_card4_title</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>≤5 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>s3_card4_score</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>e.g. 4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>s3_card4_evidence</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>s3_card4_support</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>≤20 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>s3_card4_output</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>≤10 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>s3_crosscutting</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>1 sentence</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>s3_next1</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>≤12 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>s3_next2</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>≤12 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>s3_next3</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>≤12 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>s3_footnote</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>1 line</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>s3_notes</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>Sources, one per line</t>
         </is>
@@ -6059,7 +6619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B129"/>
+  <dimension ref="A1:B172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6087,7 +6647,7 @@
         </is>
       </c>
       <c r="B3" s="16">
-        <f>MIN(12,COUNTIF(Scoring!$K$5:$K$19,"High")+COUNTIF(Scoring!$K$5:$K$19,"Medium"))</f>
+        <f>MIN(9,COUNTIF(Scoring!$K$5:$K$19,"High")+COUNTIF(Scoring!$K$5:$K$19,"Medium"))</f>
         <v/>
       </c>
     </row>
@@ -6139,7 +6699,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>{{s1_title}}</t>
+          <t>{{client_short}}</t>
         </is>
       </c>
       <c r="B8" s="8">
@@ -6150,7 +6710,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>{{s1_section}}</t>
+          <t>{{s1_title}}</t>
         </is>
       </c>
       <c r="B9" s="8">
@@ -6161,7 +6721,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>{{stat1}}</t>
+          <t>{{s1_section}}</t>
         </is>
       </c>
       <c r="B10" s="8">
@@ -6172,7 +6732,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>{{stat1_text}}</t>
+          <t>{{c1_head}}</t>
         </is>
       </c>
       <c r="B11" s="8">
@@ -6183,29 +6743,29 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>{{stat2}}</t>
+          <t>{{c1_stat}}</t>
         </is>
       </c>
       <c r="B12" s="8">
-        <f>IF(Slide_Content!$B$12="","",Slide_Content!$B$12)</f>
+        <f>IF(Slide_Content!$B$12="",TEXT(SUM(Taxonomy!$G$5:$G$19),"0"),Slide_Content!$B$12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>{{stat2_text}}</t>
+          <t>{{c1_stat_text}}</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>IF(Slide_Content!$B$13="","",Slide_Content!$B$13)</f>
+        <f>IF(Slide_Content!$B$13="",Inputs!$B$7&amp;" NBSAP commitments worth c.$"&amp;TEXT(SUM(Taxonomy!$H$5:$H$19),"0")&amp;"bn (indicative)",Slide_Content!$B$13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>{{stat3}}</t>
+          <t>{{c1_p1_lead}}</t>
         </is>
       </c>
       <c r="B14" s="8">
@@ -6216,7 +6776,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>{{stat3_text}}</t>
+          <t>{{c1_p1}}</t>
         </is>
       </c>
       <c r="B15" s="8">
@@ -6227,7 +6787,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>{{s1_context}}</t>
+          <t>{{c1_p2_lead}}</t>
         </is>
       </c>
       <c r="B16" s="8">
@@ -6238,7 +6798,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>{{s1_finding1}}</t>
+          <t>{{c1_p2}}</t>
         </is>
       </c>
       <c r="B17" s="8">
@@ -6249,7 +6809,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>{{s1_finding2}}</t>
+          <t>{{c1_p3_lead}}</t>
         </is>
       </c>
       <c r="B18" s="8">
@@ -6260,7 +6820,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>{{s1_finding3}}</t>
+          <t>{{c1_p3}}</t>
         </is>
       </c>
       <c r="B19" s="8">
@@ -6271,7 +6831,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>{{s1_priorities}}</t>
+          <t>{{c2_head}}</t>
         </is>
       </c>
       <c r="B20" s="8">
@@ -6282,7 +6842,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>{{s1_implication}}</t>
+          <t>{{c2_stat}}</t>
         </is>
       </c>
       <c r="B21" s="8">
@@ -6293,7 +6853,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>{{s1_footnote}}</t>
+          <t>{{c2_stat_text}}</t>
         </is>
       </c>
       <c r="B22" s="8">
@@ -6304,7 +6864,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>{{s1_notes}}</t>
+          <t>{{c2_p1_lead}}</t>
         </is>
       </c>
       <c r="B23" s="8">
@@ -6315,7 +6875,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>{{s2_title}}</t>
+          <t>{{c2_p1}}</t>
         </is>
       </c>
       <c r="B24" s="8">
@@ -6326,7 +6886,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>{{s2_section}}</t>
+          <t>{{c2_p2_lead}}</t>
         </is>
       </c>
       <c r="B25" s="8">
@@ -6337,7 +6897,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>{{s2_low_note}}</t>
+          <t>{{c2_p2}}</t>
         </is>
       </c>
       <c r="B26" s="8">
@@ -6348,7 +6908,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>{{s2_footnote}}</t>
+          <t>{{c2_p3_lead}}</t>
         </is>
       </c>
       <c r="B27" s="8">
@@ -6359,7 +6919,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>{{s2_notes}}</t>
+          <t>{{c2_p3}}</t>
         </is>
       </c>
       <c r="B28" s="8">
@@ -6370,7 +6930,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>{{s3_title}}</t>
+          <t>{{c3_head}}</t>
         </is>
       </c>
       <c r="B29" s="8">
@@ -6381,7 +6941,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>{{s3_section}}</t>
+          <t>{{c3_stat}}</t>
         </is>
       </c>
       <c r="B30" s="8">
@@ -6392,7 +6952,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card1_title}}</t>
+          <t>{{c3_stat_text}}</t>
         </is>
       </c>
       <c r="B31" s="8">
@@ -6403,7 +6963,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card1_score}}</t>
+          <t>{{c3_p1_lead}}</t>
         </is>
       </c>
       <c r="B32" s="8">
@@ -6414,7 +6974,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card1_evidence}}</t>
+          <t>{{c3_p1}}</t>
         </is>
       </c>
       <c r="B33" s="8">
@@ -6425,7 +6985,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card1_support}}</t>
+          <t>{{c3_p2_lead}}</t>
         </is>
       </c>
       <c r="B34" s="8">
@@ -6436,7 +6996,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card1_output}}</t>
+          <t>{{c3_p2}}</t>
         </is>
       </c>
       <c r="B35" s="8">
@@ -6447,7 +7007,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card2_title}}</t>
+          <t>{{c3_p3_lead}}</t>
         </is>
       </c>
       <c r="B36" s="8">
@@ -6458,7 +7018,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card2_score}}</t>
+          <t>{{c3_p3}}</t>
         </is>
       </c>
       <c r="B37" s="8">
@@ -6469,7 +7029,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card2_evidence}}</t>
+          <t>{{s1_found_note}}</t>
         </is>
       </c>
       <c r="B38" s="8">
@@ -6480,7 +7040,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card2_support}}</t>
+          <t>{{s1_sowhat}}</t>
         </is>
       </c>
       <c r="B39" s="8">
@@ -6491,7 +7051,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card2_output}}</t>
+          <t>{{s1_footnote}}</t>
         </is>
       </c>
       <c r="B40" s="8">
@@ -6502,7 +7062,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card3_title}}</t>
+          <t>{{s1_notes}}</t>
         </is>
       </c>
       <c r="B41" s="8">
@@ -6513,7 +7073,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card3_score}}</t>
+          <t>{{s2_title}}</t>
         </is>
       </c>
       <c r="B42" s="8">
@@ -6524,7 +7084,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card3_evidence}}</t>
+          <t>{{s2_section}}</t>
         </is>
       </c>
       <c r="B43" s="8">
@@ -6535,7 +7095,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card3_support}}</t>
+          <t>{{exp_unit}}</t>
         </is>
       </c>
       <c r="B44" s="8">
@@ -6546,7 +7106,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card3_output}}</t>
+          <t>{{t1_value}}</t>
         </is>
       </c>
       <c r="B45" s="8">
@@ -6557,7 +7117,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card4_title}}</t>
+          <t>{{t1_label}}</t>
         </is>
       </c>
       <c r="B46" s="8">
@@ -6568,7 +7128,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card4_score}}</t>
+          <t>{{t1_links}}</t>
         </is>
       </c>
       <c r="B47" s="8">
@@ -6579,7 +7139,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card4_evidence}}</t>
+          <t>{{t1_flag}}</t>
         </is>
       </c>
       <c r="B48" s="8">
@@ -6590,7 +7150,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card4_support}}</t>
+          <t>{{t2_value}}</t>
         </is>
       </c>
       <c r="B49" s="8">
@@ -6601,7 +7161,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>{{s3_card4_output}}</t>
+          <t>{{t2_label}}</t>
         </is>
       </c>
       <c r="B50" s="8">
@@ -6612,7 +7172,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>{{s3_crosscutting}}</t>
+          <t>{{t2_links}}</t>
         </is>
       </c>
       <c r="B51" s="8">
@@ -6623,7 +7183,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>{{s3_next1}}</t>
+          <t>{{t2_flag}}</t>
         </is>
       </c>
       <c r="B52" s="8">
@@ -6634,7 +7194,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>{{s3_next2}}</t>
+          <t>{{t3_value}}</t>
         </is>
       </c>
       <c r="B53" s="8">
@@ -6645,7 +7205,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>{{s3_next3}}</t>
+          <t>{{t3_label}}</t>
         </is>
       </c>
       <c r="B54" s="8">
@@ -6656,7 +7216,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>{{s3_footnote}}</t>
+          <t>{{t3_links}}</t>
         </is>
       </c>
       <c r="B55" s="8">
@@ -6667,7 +7227,7 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>{{s3_notes}}</t>
+          <t>{{t3_flag}}</t>
         </is>
       </c>
       <c r="B56" s="8">
@@ -6678,803 +7238,1276 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>{{1_name}}</t>
-        </is>
-      </c>
-      <c r="B57" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t4_value}}</t>
+        </is>
+      </c>
+      <c r="B57" s="8">
+        <f>IF(Slide_Content!$B$57="","",Slide_Content!$B$57)</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>{{1_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B58" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{t4_label}}</t>
+        </is>
+      </c>
+      <c r="B58" s="8">
+        <f>IF(Slide_Content!$B$58="","",Slide_Content!$B$58)</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>{{1_exp}}</t>
-        </is>
-      </c>
-      <c r="B59" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t4_links}}</t>
+        </is>
+      </c>
+      <c r="B59" s="8">
+        <f>IF(Slide_Content!$B$59="","",Slide_Content!$B$59)</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>{{1s}}</t>
-        </is>
-      </c>
-      <c r="B60" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{t4_flag}}</t>
+        </is>
+      </c>
+      <c r="B60" s="8">
+        <f>IF(Slide_Content!$B$60="","",Slide_Content!$B$60)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>{{1t}}</t>
-        </is>
-      </c>
-      <c r="B61" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t5_value}}</t>
+        </is>
+      </c>
+      <c r="B61" s="8">
+        <f>IF(Slide_Content!$B$61="","",Slide_Content!$B$61)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>{{1_evid}}</t>
-        </is>
-      </c>
-      <c r="B62" s="19">
-        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t5_label}}</t>
+        </is>
+      </c>
+      <c r="B62" s="8">
+        <f>IF(Slide_Content!$B$62="","",Slide_Content!$B$62)</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>{{2_name}}</t>
-        </is>
-      </c>
-      <c r="B63" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t5_links}}</t>
+        </is>
+      </c>
+      <c r="B63" s="8">
+        <f>IF(Slide_Content!$B$63="","",Slide_Content!$B$63)</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>{{2_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B64" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{t5_flag}}</t>
+        </is>
+      </c>
+      <c r="B64" s="8">
+        <f>IF(Slide_Content!$B$64="","",Slide_Content!$B$64)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>{{2_exp}}</t>
-        </is>
-      </c>
-      <c r="B65" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t6_value}}</t>
+        </is>
+      </c>
+      <c r="B65" s="8">
+        <f>IF(Slide_Content!$B$65="","",Slide_Content!$B$65)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>{{2s}}</t>
-        </is>
-      </c>
-      <c r="B66" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{t6_label}}</t>
+        </is>
+      </c>
+      <c r="B66" s="8">
+        <f>IF(Slide_Content!$B$66="","",Slide_Content!$B$66)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>{{2t}}</t>
-        </is>
-      </c>
-      <c r="B67" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t6_links}}</t>
+        </is>
+      </c>
+      <c r="B67" s="8">
+        <f>IF(Slide_Content!$B$67="","",Slide_Content!$B$67)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>{{2_evid}}</t>
-        </is>
-      </c>
-      <c r="B68" s="19">
-        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{t6_flag}}</t>
+        </is>
+      </c>
+      <c r="B68" s="8">
+        <f>IF(Slide_Content!$B$68="","",Slide_Content!$B$68)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>{{3_name}}</t>
-        </is>
-      </c>
-      <c r="B69" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s2_sowhat}}</t>
+        </is>
+      </c>
+      <c r="B69" s="8">
+        <f>IF(Slide_Content!$B$69="","",Slide_Content!$B$69)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>{{3_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B70" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{s2_footnote}}</t>
+        </is>
+      </c>
+      <c r="B70" s="8">
+        <f>IF(Slide_Content!$B$70="","",Slide_Content!$B$70)</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>{{3_exp}}</t>
-        </is>
-      </c>
-      <c r="B71" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s2_notes}}</t>
+        </is>
+      </c>
+      <c r="B71" s="8">
+        <f>IF(Slide_Content!$B$71="","",Slide_Content!$B$71)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>{{3s}}</t>
-        </is>
-      </c>
-      <c r="B72" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{s3_title}}</t>
+        </is>
+      </c>
+      <c r="B72" s="8">
+        <f>IF(Slide_Content!$B$72="","",Slide_Content!$B$72)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>{{3t}}</t>
-        </is>
-      </c>
-      <c r="B73" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_section}}</t>
+        </is>
+      </c>
+      <c r="B73" s="8">
+        <f>IF(Slide_Content!$B$73="","",Slide_Content!$B$73)</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>{{3_evid}}</t>
-        </is>
-      </c>
-      <c r="B74" s="19">
-        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card1_title}}</t>
+        </is>
+      </c>
+      <c r="B74" s="8">
+        <f>IF(Slide_Content!$B$74="","",Slide_Content!$B$74)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>{{4_name}}</t>
-        </is>
-      </c>
-      <c r="B75" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card1_score}}</t>
+        </is>
+      </c>
+      <c r="B75" s="8">
+        <f>IF(Slide_Content!$B$75="","",Slide_Content!$B$75)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>{{4_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B76" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{s3_card1_evidence}}</t>
+        </is>
+      </c>
+      <c r="B76" s="8">
+        <f>IF(Slide_Content!$B$76="","",Slide_Content!$B$76)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>{{4_exp}}</t>
-        </is>
-      </c>
-      <c r="B77" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card1_support}}</t>
+        </is>
+      </c>
+      <c r="B77" s="8">
+        <f>IF(Slide_Content!$B$77="","",Slide_Content!$B$77)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>{{4s}}</t>
-        </is>
-      </c>
-      <c r="B78" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{s3_card1_output}}</t>
+        </is>
+      </c>
+      <c r="B78" s="8">
+        <f>IF(Slide_Content!$B$78="","",Slide_Content!$B$78)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>{{4t}}</t>
-        </is>
-      </c>
-      <c r="B79" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card2_title}}</t>
+        </is>
+      </c>
+      <c r="B79" s="8">
+        <f>IF(Slide_Content!$B$79="","",Slide_Content!$B$79)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>{{4_evid}}</t>
-        </is>
-      </c>
-      <c r="B80" s="19">
-        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card2_score}}</t>
+        </is>
+      </c>
+      <c r="B80" s="8">
+        <f>IF(Slide_Content!$B$80="","",Slide_Content!$B$80)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>{{5_name}}</t>
-        </is>
-      </c>
-      <c r="B81" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card2_evidence}}</t>
+        </is>
+      </c>
+      <c r="B81" s="8">
+        <f>IF(Slide_Content!$B$81="","",Slide_Content!$B$81)</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>{{5_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B82" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{s3_card2_support}}</t>
+        </is>
+      </c>
+      <c r="B82" s="8">
+        <f>IF(Slide_Content!$B$82="","",Slide_Content!$B$82)</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>{{5_exp}}</t>
-        </is>
-      </c>
-      <c r="B83" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card2_output}}</t>
+        </is>
+      </c>
+      <c r="B83" s="8">
+        <f>IF(Slide_Content!$B$83="","",Slide_Content!$B$83)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>{{5s}}</t>
-        </is>
-      </c>
-      <c r="B84" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{s3_card3_title}}</t>
+        </is>
+      </c>
+      <c r="B84" s="8">
+        <f>IF(Slide_Content!$B$84="","",Slide_Content!$B$84)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>{{5t}}</t>
-        </is>
-      </c>
-      <c r="B85" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card3_score}}</t>
+        </is>
+      </c>
+      <c r="B85" s="8">
+        <f>IF(Slide_Content!$B$85="","",Slide_Content!$B$85)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>{{5_evid}}</t>
-        </is>
-      </c>
-      <c r="B86" s="19">
-        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card3_evidence}}</t>
+        </is>
+      </c>
+      <c r="B86" s="8">
+        <f>IF(Slide_Content!$B$86="","",Slide_Content!$B$86)</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>{{6_name}}</t>
-        </is>
-      </c>
-      <c r="B87" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card3_support}}</t>
+        </is>
+      </c>
+      <c r="B87" s="8">
+        <f>IF(Slide_Content!$B$87="","",Slide_Content!$B$87)</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>{{6_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B88" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{s3_card3_output}}</t>
+        </is>
+      </c>
+      <c r="B88" s="8">
+        <f>IF(Slide_Content!$B$88="","",Slide_Content!$B$88)</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>{{6_exp}}</t>
-        </is>
-      </c>
-      <c r="B89" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card4_title}}</t>
+        </is>
+      </c>
+      <c r="B89" s="8">
+        <f>IF(Slide_Content!$B$89="","",Slide_Content!$B$89)</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>{{6s}}</t>
-        </is>
-      </c>
-      <c r="B90" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{s3_card4_score}}</t>
+        </is>
+      </c>
+      <c r="B90" s="8">
+        <f>IF(Slide_Content!$B$90="","",Slide_Content!$B$90)</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>{{6t}}</t>
-        </is>
-      </c>
-      <c r="B91" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card4_evidence}}</t>
+        </is>
+      </c>
+      <c r="B91" s="8">
+        <f>IF(Slide_Content!$B$91="","",Slide_Content!$B$91)</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>{{6_evid}}</t>
-        </is>
-      </c>
-      <c r="B92" s="19">
-        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card4_support}}</t>
+        </is>
+      </c>
+      <c r="B92" s="8">
+        <f>IF(Slide_Content!$B$92="","",Slide_Content!$B$92)</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>{{7_name}}</t>
-        </is>
-      </c>
-      <c r="B93" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_card4_output}}</t>
+        </is>
+      </c>
+      <c r="B93" s="8">
+        <f>IF(Slide_Content!$B$93="","",Slide_Content!$B$93)</f>
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>{{7_nbsap}}</t>
-        </is>
-      </c>
-      <c r="B94" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+          <t>{{s3_crosscutting}}</t>
+        </is>
+      </c>
+      <c r="B94" s="8">
+        <f>IF(Slide_Content!$B$94="","",Slide_Content!$B$94)</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>{{7_exp}}</t>
-        </is>
-      </c>
-      <c r="B95" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_next1}}</t>
+        </is>
+      </c>
+      <c r="B95" s="8">
+        <f>IF(Slide_Content!$B$95="","",Slide_Content!$B$95)</f>
         <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>{{7s}}</t>
-        </is>
-      </c>
-      <c r="B96" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+          <t>{{s3_next2}}</t>
+        </is>
+      </c>
+      <c r="B96" s="8">
+        <f>IF(Slide_Content!$B$96="","",Slide_Content!$B$96)</f>
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>{{7t}}</t>
-        </is>
-      </c>
-      <c r="B97" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_next3}}</t>
+        </is>
+      </c>
+      <c r="B97" s="8">
+        <f>IF(Slide_Content!$B$97="","",Slide_Content!$B$97)</f>
         <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>{{7_evid}}</t>
-        </is>
-      </c>
-      <c r="B98" s="19">
-        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_footnote}}</t>
+        </is>
+      </c>
+      <c r="B98" s="8">
+        <f>IF(Slide_Content!$B$98="","",Slide_Content!$B$98)</f>
         <v/>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>{{8_name}}</t>
-        </is>
-      </c>
-      <c r="B99" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+          <t>{{s3_notes}}</t>
+        </is>
+      </c>
+      <c r="B99" s="8">
+        <f>IF(Slide_Content!$B$99="","",Slide_Content!$B$99)</f>
         <v/>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>{{8_nbsap}}</t>
+          <t>{{1_name}}</t>
         </is>
       </c>
       <c r="B100" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>{{8_exp}}</t>
+          <t>{{1_nbsap}}</t>
         </is>
       </c>
       <c r="B101" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>{{8s}}</t>
+          <t>{{1_exp}}</t>
         </is>
       </c>
       <c r="B102" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>{{8t}}</t>
+          <t>{{1s}}</t>
         </is>
       </c>
       <c r="B103" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>{{8_evid}}</t>
+          <t>{{1t}}</t>
         </is>
       </c>
       <c r="B104" s="19">
-        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>{{9_name}}</t>
+          <t>{{1_evid}}</t>
         </is>
       </c>
       <c r="B105" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(1&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>{{9_nbsap}}</t>
+          <t>{{2_name}}</t>
         </is>
       </c>
       <c r="B106" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>{{9_exp}}</t>
+          <t>{{2_nbsap}}</t>
         </is>
       </c>
       <c r="B107" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>{{9s}}</t>
+          <t>{{2_exp}}</t>
         </is>
       </c>
       <c r="B108" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>{{9t}}</t>
+          <t>{{2s}}</t>
         </is>
       </c>
       <c r="B109" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>{{9_evid}}</t>
+          <t>{{2t}}</t>
         </is>
       </c>
       <c r="B110" s="19">
-        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>{{10_name}}</t>
+          <t>{{2_evid}}</t>
         </is>
       </c>
       <c r="B111" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(2&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>{{10_nbsap}}</t>
+          <t>{{3_name}}</t>
         </is>
       </c>
       <c r="B112" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>{{10_exp}}</t>
+          <t>{{3_nbsap}}</t>
         </is>
       </c>
       <c r="B113" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>{{10s}}</t>
+          <t>{{3_exp}}</t>
         </is>
       </c>
       <c r="B114" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>{{10t}}</t>
+          <t>{{3s}}</t>
         </is>
       </c>
       <c r="B115" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>{{10_evid}}</t>
+          <t>{{3t}}</t>
         </is>
       </c>
       <c r="B116" s="19">
-        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>{{11_name}}</t>
+          <t>{{3_evid}}</t>
         </is>
       </c>
       <c r="B117" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(3&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>{{11_nbsap}}</t>
+          <t>{{4_name}}</t>
         </is>
       </c>
       <c r="B118" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>{{11_exp}}</t>
+          <t>{{4_nbsap}}</t>
         </is>
       </c>
       <c r="B119" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>{{11s}}</t>
+          <t>{{4_exp}}</t>
         </is>
       </c>
       <c r="B120" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>{{11t}}</t>
+          <t>{{4s}}</t>
         </is>
       </c>
       <c r="B121" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>{{11_evid}}</t>
+          <t>{{4t}}</t>
         </is>
       </c>
       <c r="B122" s="19">
-        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>{{12_name}}</t>
+          <t>{{4_evid}}</t>
         </is>
       </c>
       <c r="B123" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(4&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>{{12_nbsap}}</t>
+          <t>{{5_name}}</t>
         </is>
       </c>
       <c r="B124" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>{{12_exp}}</t>
+          <t>{{5_nbsap}}</t>
         </is>
       </c>
       <c r="B125" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(5&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>{{12s}}</t>
+          <t>{{5_exp}}</t>
         </is>
       </c>
       <c r="B126" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>{{12t}}</t>
+          <t>{{5s}}</t>
         </is>
       </c>
       <c r="B127" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(5&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>{{12_evid}}</t>
+          <t>{{5t}}</t>
         </is>
       </c>
       <c r="B128" s="19">
-        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
+          <t>{{5_evid}}</t>
+        </is>
+      </c>
+      <c r="B129" s="19">
+        <f>IF(5&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>{{6_name}}</t>
+        </is>
+      </c>
+      <c r="B130" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>{{6_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B131" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>{{6_exp}}</t>
+        </is>
+      </c>
+      <c r="B132" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>{{6s}}</t>
+        </is>
+      </c>
+      <c r="B133" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>{{6t}}</t>
+        </is>
+      </c>
+      <c r="B134" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>{{6_evid}}</t>
+        </is>
+      </c>
+      <c r="B135" s="19">
+        <f>IF(6&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>{{7_name}}</t>
+        </is>
+      </c>
+      <c r="B136" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>{{7_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B137" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>{{7_exp}}</t>
+        </is>
+      </c>
+      <c r="B138" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>{{7s}}</t>
+        </is>
+      </c>
+      <c r="B139" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>{{7t}}</t>
+        </is>
+      </c>
+      <c r="B140" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>{{7_evid}}</t>
+        </is>
+      </c>
+      <c r="B141" s="19">
+        <f>IF(7&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>{{8_name}}</t>
+        </is>
+      </c>
+      <c r="B142" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>{{8_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B143" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>{{8_exp}}</t>
+        </is>
+      </c>
+      <c r="B144" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>{{8s}}</t>
+        </is>
+      </c>
+      <c r="B145" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>{{8t}}</t>
+        </is>
+      </c>
+      <c r="B146" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>{{8_evid}}</t>
+        </is>
+      </c>
+      <c r="B147" s="19">
+        <f>IF(8&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>{{9_name}}</t>
+        </is>
+      </c>
+      <c r="B148" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>{{9_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B149" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>{{9_exp}}</t>
+        </is>
+      </c>
+      <c r="B150" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>{{9s}}</t>
+        </is>
+      </c>
+      <c r="B151" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>{{9t}}</t>
+        </is>
+      </c>
+      <c r="B152" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>{{9_evid}}</t>
+        </is>
+      </c>
+      <c r="B153" s="19">
+        <f>IF(9&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>{{10_name}}</t>
+        </is>
+      </c>
+      <c r="B154" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>{{10_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B155" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>{{10_exp}}</t>
+        </is>
+      </c>
+      <c r="B156" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>{{10s}}</t>
+        </is>
+      </c>
+      <c r="B157" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>{{10t}}</t>
+        </is>
+      </c>
+      <c r="B158" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>{{10_evid}}</t>
+        </is>
+      </c>
+      <c r="B159" s="19">
+        <f>IF(10&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>{{11_name}}</t>
+        </is>
+      </c>
+      <c r="B160" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>{{11_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B161" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>{{11_exp}}</t>
+        </is>
+      </c>
+      <c r="B162" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>{{11s}}</t>
+        </is>
+      </c>
+      <c r="B163" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>{{11t}}</t>
+        </is>
+      </c>
+      <c r="B164" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>{{11_evid}}</t>
+        </is>
+      </c>
+      <c r="B165" s="19">
+        <f>IF(11&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>{{12_name}}</t>
+        </is>
+      </c>
+      <c r="B166" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>{{12_nbsap}}</t>
+        </is>
+      </c>
+      <c r="B167" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(IF(INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))=0,"– | 0",IF(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&lt;0.1,"&lt;$0.1bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"$"&amp;TEXT(INDEX(Taxonomy!$H$5:$H$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0)),"0.0")&amp;"bn | "&amp;INDEX(Taxonomy!$G$5:$G$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>{{12_exp}}</t>
+        </is>
+      </c>
+      <c r="B168" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$U$5:$U$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>{{12s}}</t>
+        </is>
+      </c>
+      <c r="B169" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0")&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>{{12t}}</t>
+        </is>
+      </c>
+      <c r="B170" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$K$5:$K$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>{{12_evid}}</t>
+        </is>
+      </c>
+      <c r="B171" s="19">
+        <f>IF(12&gt;$B$3,"",IFERROR(INDEX(Scoring!$T$5:$T$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;"",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
           <t>{{low_list}}</t>
         </is>
       </c>
-      <c r="B129" s="19">
-        <f>IF(1&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(1&lt;15,"  |  ",""),"")&amp;IF(2&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(2&lt;15,"  |  ",""),"")&amp;IF(3&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(3&lt;15,"  |  ",""),"")&amp;IF(4&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(4&lt;15,"  |  ",""),"")&amp;IF(5&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(5&lt;15,"  |  ",""),"")&amp;IF(6&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(6&lt;15,"  |  ",""),"")&amp;IF(7&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(7&lt;15,"  |  ",""),"")&amp;IF(8&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(8&lt;15,"  |  ",""),"")&amp;IF(9&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(9&lt;15,"  |  ",""),"")&amp;IF(10&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(10,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(10&lt;15,"  |  ",""),"")&amp;IF(11&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(11,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(11&lt;15,"  |  ",""),"")&amp;IF(12&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(12,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(12&lt;15,"  |  ",""),"")&amp;IF(13&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(13,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(13,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(13&lt;15,"  |  ",""),"")&amp;IF(14&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(14,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(14,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(14&lt;15,"  |  ",""),"")&amp;IF(15&gt;$B$3,IFERROR(INDEX(Scoring!$D$5:$D$19,MATCH(15,Scoring!$A$5:$A$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(15,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(15&lt;15,"  |  ",""),"")</f>
+      <c r="B172" s="19">
+        <f>IF(1&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(1,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(1&lt;15,", ",""),"")&amp;IF(2&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(2,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(2&lt;15,", ",""),"")&amp;IF(3&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(3,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(3&lt;15,", ",""),"")&amp;IF(4&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(4,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(4&lt;15,", ",""),"")&amp;IF(5&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(5,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(5&lt;15,", ",""),"")&amp;IF(6&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(6,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(6&lt;15,", ",""),"")&amp;IF(7&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(7,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(7&lt;15,", ",""),"")&amp;IF(8&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(8,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(8&lt;15,", ",""),"")&amp;IF(9&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(9,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(9&lt;15,", ",""),"")&amp;IF(10&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(10,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(10,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(10&lt;15,", ",""),"")&amp;IF(11&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(11,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(11,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(11&lt;15,", ",""),"")&amp;IF(12&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(12,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(12,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(12&lt;15,", ",""),"")&amp;IF(13&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(13,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(13,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(13&lt;15,", ",""),"")&amp;IF(14&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(14,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(14,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(14&lt;15,", ",""),"")&amp;IF(15&gt;$B$3,IFERROR(INDEX(Taxonomy!$M$5:$M$19,MATCH(INDEX(Scoring!$B$5:$B$19,MATCH(15,Scoring!$A$5:$A$19,0)),Taxonomy!$C$5:$C$19,0))&amp;" "&amp;TEXT(INDEX(Scoring!$J$5:$J$19,MATCH(15,Scoring!$A$5:$A$19,0)),"0.0"),"")&amp;IF(15&lt;15,", ",""),"")</f>
         <v/>
       </c>
     </row>
@@ -7484,6 +8517,182 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Chart data for page 3 (paste into the chart: right-click &gt; Edit Data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Copy A4:C13 and paste over the chart data sheet in PowerPoint (cell A1). Blank rows mean fewer than 9 High/Medium priorities: delete those rows in the chart data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19">
+        <f>IF(1&gt;Deck_Tokens!$B$3,"",1&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(1,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B5" s="25">
+        <f>IF(1&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(1,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C5" s="25">
+        <f>IF(1&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(1,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(1,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19">
+        <f>IF(2&gt;Deck_Tokens!$B$3,"",2&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(2,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B6" s="25">
+        <f>IF(2&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(2,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C6" s="25">
+        <f>IF(2&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(2,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(2,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19">
+        <f>IF(3&gt;Deck_Tokens!$B$3,"",3&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(3,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B7" s="25">
+        <f>IF(3&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(3,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C7" s="25">
+        <f>IF(3&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(3,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(3,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19">
+        <f>IF(4&gt;Deck_Tokens!$B$3,"",4&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(4,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B8" s="25">
+        <f>IF(4&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(4,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C8" s="25">
+        <f>IF(4&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(4,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(4,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19">
+        <f>IF(5&gt;Deck_Tokens!$B$3,"",5&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(5,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B9" s="25">
+        <f>IF(5&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(5,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C9" s="25">
+        <f>IF(5&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(5,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(5,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19">
+        <f>IF(6&gt;Deck_Tokens!$B$3,"",6&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(6,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B10" s="25">
+        <f>IF(6&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(6,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C10" s="25">
+        <f>IF(6&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(6,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(6,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19">
+        <f>IF(7&gt;Deck_Tokens!$B$3,"",7&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(7,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B11" s="25">
+        <f>IF(7&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(7,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C11" s="25">
+        <f>IF(7&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(7,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(7,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19">
+        <f>IF(8&gt;Deck_Tokens!$B$3,"",8&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(8,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B12" s="25">
+        <f>IF(8&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(8,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C12" s="25">
+        <f>IF(8&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(8,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(8,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19">
+        <f>IF(9&gt;Deck_Tokens!$B$3,"",9&amp;"   "&amp;INDEX(Scoring!$D$5:$D$19,MATCH(9,Scoring!$A$5:$A$19,0)))</f>
+        <v/>
+      </c>
+      <c r="B13" s="25">
+        <f>IF(9&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(9,Scoring!$A$5:$A$19,0))="High",INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C13" s="25">
+        <f>IF(9&gt;Deck_Tokens!$B$3,"",IF(INDEX(Scoring!$K$5:$K$19,MATCH(9,Scoring!$A$5:$A$19,0))="Medium",INDEX(Scoring!$J$5:$J$19,MATCH(9,Scoring!$A$5:$A$19,0)),""))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10506,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10521,6 +11730,7 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10598,6 +11808,11 @@
           <t>NBSAP target link (selected country)</t>
         </is>
       </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Short name (slides)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -10654,6 +11869,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C5),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Water usage</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -10710,6 +11930,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C6),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>Water quality</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -10766,6 +11991,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C7),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>Water availability</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -10822,6 +12052,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C8),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>Forestry</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -10878,6 +12113,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C9),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -10934,6 +12174,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C10),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>Fisheries</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -10990,6 +12235,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C11),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>Nature-positive buildings</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -11046,6 +12296,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C12),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>Green-blue infrastructure</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -11102,6 +12357,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C13),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>Habitat protection</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -11158,6 +12418,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C14),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>Risk reduction</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -11214,6 +12479,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C15),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>Flood mitigation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -11270,6 +12540,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C16),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>Adaptation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -11326,6 +12601,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C17),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -11382,6 +12662,11 @@
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C18),0),0)+4),"[to confirm]")</f>
         <v/>
       </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>Waste and circular economy</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -11437,6 +12722,11 @@
       <c r="L19" s="8">
         <f>IFERROR(INDEX(NBSAP_Targets!$C:$C,MATCH(1,INDEX((NBSAP_Targets!$A$5:$A$500=Inputs!$B$6)*(NBSAP_Targets!$B$5:$B$500=C19),0),0)+4),"[to confirm]")</f>
         <v/>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>Air and noise</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>